<commit_message>
HPを更新（homepage-next から publish_to_pages.py で反映）
</commit_message>
<xml_diff>
--- a/jigyosho/izumo_kaigo_list.xlsx
+++ b/jigyosho/izumo_kaigo_list.xlsx
@@ -14012,7 +14012,11 @@
           <t>3260490267</t>
         </is>
       </c>
-      <c r="K66" s="6" t="inlineStr"/>
+      <c r="K66" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lifecreate-grow.com/grow</t>
+        </is>
+      </c>
       <c r="L66" s="6" t="inlineStr"/>
     </row>
     <row r="67">
@@ -33320,260 +33324,261 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K126" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K143" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K144" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K146" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K148" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K149" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K150" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K151" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K152" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K156" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K157" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K158" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K161" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K163" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K165" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K166" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K168" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K169" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K170" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K174" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K176" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K177" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K178" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K179" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K180" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K181" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K182" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K183" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K184" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K185" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K186" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K187" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K189" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K190" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K191" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K192" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K193" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K194" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K197" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K198" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K199" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K200" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K201" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K202" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K203" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K204" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L204" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K205" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L205" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K206" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K207" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K208" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K211" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L211" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K212" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K213" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K214" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K216" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K217" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K220" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K221" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K224" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K226" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K227" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K228" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K235" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L235" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K236" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K239" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L239" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K240" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L240" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K241" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K242" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K243" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K244" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K245" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K246" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K247" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K248" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K249" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K250" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L250" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K251" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K252" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K254" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K255" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K259" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K261" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K262" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K263" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K265" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K266" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K267" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K271" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K273" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K279" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K282" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K288" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K292" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K293" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K296" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K304" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K305" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K306" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K307" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K310" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K311" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K313" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K314" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K316" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K320" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K321" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K322" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K323" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K325" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K326" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K327" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K328" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K331" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K332" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K336" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K337" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K338" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K339" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K340" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K341" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K342" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K343" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L343" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K345" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K346" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K347" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K348" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L348" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K349" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L349" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K350" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K351" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K352" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K353" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K354" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K355" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L355" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K356" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K357" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K358" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L358" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K359" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K360" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K361" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K362" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K363" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K364" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K365" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K366" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K367" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K369" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K370" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K371" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K372" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K373" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K374" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K375" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K378" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K379" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K380" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K384" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K385" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K388" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K389" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L389" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K390" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L390" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K391" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K392" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K393" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K394" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K399" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K400" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K401" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K402" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K403" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K405" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K406" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K407" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K408" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K409" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K410" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K413" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K416" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K418" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K419" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K420" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K421" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K426" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L426" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K427" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L427" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K428" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K429" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K430" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K431" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K433" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K435" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K126" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K143" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K144" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K146" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K148" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K149" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K150" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K151" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K152" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K156" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K157" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K158" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K161" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K163" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K165" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K166" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K168" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K169" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K170" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K174" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K176" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K177" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K178" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K179" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K180" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K181" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K182" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K183" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K184" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K185" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K186" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K187" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K189" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K190" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K191" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K192" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K193" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K194" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K197" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K198" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K199" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K200" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K201" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K202" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K203" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K204" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L204" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K205" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L205" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K206" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K207" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K208" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K211" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L211" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K212" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K213" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K214" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K216" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K217" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K220" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K221" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K224" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K226" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K227" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K228" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K235" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L235" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K236" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K239" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L239" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K240" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L240" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K241" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K242" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K243" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K244" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K245" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K246" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K247" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K248" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K249" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K250" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L250" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K251" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K252" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K254" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K255" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K259" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K261" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K262" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K263" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K265" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K266" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K267" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K271" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K273" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K279" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K282" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K288" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K292" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K293" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K296" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K304" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K305" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K306" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K307" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K310" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K311" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K313" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K314" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K316" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K320" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K321" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K322" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K323" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K325" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K326" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K327" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K328" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K331" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K332" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K336" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K337" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K338" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K339" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K340" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K341" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K342" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K343" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L343" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K345" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K346" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K347" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K348" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L348" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K349" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L349" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K350" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K351" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K352" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K353" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K354" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K355" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L355" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K356" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K357" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K358" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L358" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K359" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K360" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K361" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K362" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K363" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K364" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K365" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K366" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K367" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K369" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K370" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K371" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K372" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K373" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K374" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K375" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K378" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K379" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K380" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K384" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K385" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K388" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K389" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L389" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K390" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L390" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K391" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K392" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K393" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K394" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K399" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K400" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K401" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K402" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K403" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K405" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K406" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K407" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K408" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K409" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K410" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K413" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K416" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K418" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K419" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K420" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K421" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K426" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L426" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K427" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L427" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K428" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K429" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K430" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K431" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K433" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K435" r:id="rId287"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -41289,7 +41294,11 @@
           <t>3260490267</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lifecreate-grow.com/grow</t>
+        </is>
+      </c>
       <c r="K10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
@@ -42463,13 +42472,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>